<commit_message>
운동프로그램 갱신 2026-08-10  1:10:22.33
</commit_message>
<xml_diff>
--- a/운동프로그램_6일_v3.xlsx
+++ b/운동프로그램_6일_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D7F24BC338148AA2A1BB93A051E4A7F951AADFBD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_D7F24BC338148AA2A1BB93A051E4A7F951AADFBD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEF8CB0E-C159-4275-A550-D973AA7143A9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18390" yWindow="1380" windowWidth="17670" windowHeight="18480" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="620">
   <si>
     <t>금요일 — 밀기 B (수직)</t>
   </si>
@@ -474,18 +474,12 @@
     <t>1~2주</t>
   </si>
   <si>
-    <t>폼 학습 구간. 가볍다고 느껴야 정상</t>
-  </si>
-  <si>
     <t>2단계</t>
   </si>
   <si>
     <t>3~4주</t>
   </si>
   <si>
-    <t>건·인대 적응. 여기서 팔꿈치·어깨 앞쪽 통증이 나오면 계수를 내린다</t>
-  </si>
-  <si>
     <t>본구간</t>
   </si>
   <si>
@@ -549,9 +543,6 @@
     <t>운동 프로그램 — 주 6일 (당기기 · 밀기 · 하체 × 2)</t>
   </si>
   <si>
-    <t>적용 시기: 재택 근무 기간 (~9월)  |  주 6일 / 1일 1세션  |  1~4주는 볼륨램프 시트의 계수 적용</t>
-  </si>
-  <si>
     <t>요일</t>
   </si>
   <si>
@@ -1897,13 +1888,774 @@
   </si>
   <si>
     <t>· 쌓는 시기와 지키는 시기는 다르게 설계해야 한다.</t>
+  </si>
+  <si>
+    <t>2026-08-10 해제 — 계수 0.5 → 1. 되살리려면 여기 C9에 0.5를 다시 입력</t>
+    <phoneticPr fontId="27" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-08-10 해제 — 계수 0.7 → 1. 되살리려면 여기 C10에 0.7을 다시 입력</t>
+    <phoneticPr fontId="27" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>현재</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>상태</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (2026-08-10) — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>램프</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>해제됨</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>· C9 · C10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>바꿔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>주차부터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>볼륨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 100%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>간다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>. J</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>열</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>이번</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>주</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>세트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) = E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>열</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>세트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>위</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>논리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>사용법</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>램프를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>켰을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>때의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>근거이며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>기록용으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>남겨둔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>것이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>되살리려면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> C9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 0.5, C10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 0.7. J</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>열과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>앱이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>자동으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>따라온다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>적용 시기: 재택 근무 기간 (~9월)  |  주 6일 / 1일 1세션  |  1주차부터 설계 볼륨 100% (볼륨램프 해제)</t>
+    <phoneticPr fontId="27" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2103,6 +2855,19 @@
       <family val="3"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -2169,7 +2934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2356,6 +3121,7 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -3177,12 +3943,12 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
@@ -3190,19 +3956,19 @@
         <v>14</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>377</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>378</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
@@ -3225,7 +3991,7 @@
         <v>충분</v>
       </c>
       <c r="F5" s="56" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1">
@@ -3248,12 +4014,12 @@
         <v>충분</v>
       </c>
       <c r="F6" s="56" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
       <c r="A7" s="56" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B7" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A7)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A7)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A7)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A7)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A7)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A7)</f>
@@ -3271,7 +4037,7 @@
         <v>충분</v>
       </c>
       <c r="F7" s="56" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1">
@@ -3294,12 +4060,12 @@
         <v>충분</v>
       </c>
       <c r="F8" s="56" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1">
       <c r="A9" s="56" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B9" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A9)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A9)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A9)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A9)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A9)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A9)</f>
@@ -3317,12 +4083,12 @@
         <v>충분</v>
       </c>
       <c r="F9" s="56" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
       <c r="A10" s="56" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B10" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A10)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A10)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A10)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A10)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A10)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A10)</f>
@@ -3340,7 +4106,7 @@
         <v>충분</v>
       </c>
       <c r="F10" s="56" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
@@ -3363,7 +4129,7 @@
         <v>충분</v>
       </c>
       <c r="F11" s="56" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
@@ -3386,7 +4152,7 @@
         <v>충분</v>
       </c>
       <c r="F12" s="56" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1">
@@ -3409,12 +4175,12 @@
         <v>충분</v>
       </c>
       <c r="F13" s="56" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15" customHeight="1">
       <c r="A14" s="56" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B14" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A14)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A14)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A14)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A14)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A14)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A14)</f>
@@ -3432,12 +4198,12 @@
         <v>충분</v>
       </c>
       <c r="F14" s="56" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15" customHeight="1">
       <c r="A15" s="56" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B15" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A15)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A15)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A15)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A15)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A15)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A15)</f>
@@ -3455,12 +4221,12 @@
         <v>충분</v>
       </c>
       <c r="F15" s="56" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" customHeight="1">
       <c r="A16" s="56" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B16" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A16)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A16)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A16)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A16)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A16)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A16)</f>
@@ -3478,12 +4244,12 @@
         <v>충분</v>
       </c>
       <c r="F16" s="56" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1">
       <c r="A17" s="56" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B17" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A17)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A17)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A17)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A17)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A17)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A17)</f>
@@ -3501,12 +4267,12 @@
         <v>하한</v>
       </c>
       <c r="F17" s="56" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1">
       <c r="A18" s="56" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B18" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A18)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A18)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A18)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A18)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A18)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A18)</f>
@@ -3524,12 +4290,12 @@
         <v>하한</v>
       </c>
       <c r="F18" s="56" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15" customHeight="1">
       <c r="A19" s="56" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B19" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A19)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A19)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A19)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A19)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A19)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A19)</f>
@@ -3547,7 +4313,7 @@
         <v>충분</v>
       </c>
       <c r="F19" s="56" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15" customHeight="1">
@@ -3570,12 +4336,12 @@
         <v>충분</v>
       </c>
       <c r="F20" s="56" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15" customHeight="1">
       <c r="A21" s="56" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B21" s="7">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A21)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A21)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A21)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A21)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A21)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A21)</f>
@@ -3593,12 +4359,12 @@
         <v>충분</v>
       </c>
       <c r="F21" s="56" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="16.5" customHeight="1">
       <c r="A22" s="56" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B22" s="58">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A22)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A22)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A22)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A22)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A22)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A22)</f>
@@ -3616,12 +4382,12 @@
         <v>충분</v>
       </c>
       <c r="F22" s="56" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="24" customHeight="1">
       <c r="A23" s="56" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B23" s="58">
         <f>SUMIFS(월_당기기A!$E:$E,월_당기기A!$C:$C,$A23)+SUMIFS(화_밀기A!$E:$E,화_밀기A!$C:$C,$A23)+SUMIFS(수_하체A!$E:$E,수_하체A!$C:$C,$A23)+SUMIFS(목_당기기B!$E:$E,목_당기기B!$C:$C,$A23)+SUMIFS(금_밀기B!$E:$E,금_밀기B!$C:$C,$A23)+SUMIFS(토_하체B!$E:$E,토_하체B!$C:$C,$A23)</f>
@@ -3639,12 +4405,12 @@
         <v>하한</v>
       </c>
       <c r="F23" s="56" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15" customHeight="1">
       <c r="A24" s="59" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="B24" s="15">
         <f>SUM(B5:B23)</f>
@@ -3657,22 +4423,22 @@
     </row>
     <row r="25" spans="1:6" ht="36" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15" customHeight="1">
       <c r="A26" s="11" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.5" customHeight="1">
       <c r="A27" s="11" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="36" customHeight="1">
       <c r="A28" s="11" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="48" customHeight="1">
@@ -3680,22 +4446,22 @@
     </row>
     <row r="30" spans="1:6" ht="48" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16.5" customHeight="1">
       <c r="A32" s="11" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="48" customHeight="1">
       <c r="A33" s="11" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="48" customHeight="1">
@@ -3703,53 +4469,53 @@
     </row>
     <row r="35" spans="1:1" ht="15" customHeight="1">
       <c r="A35" s="13" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="48" customHeight="1">
       <c r="A36" s="11" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="77.25" customHeight="1">
       <c r="A37" s="11" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="48" customHeight="1">
       <c r="A38" s="61" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="39" customHeight="1">
       <c r="A39" s="11" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="45" customHeight="1"/>
     <row r="41" spans="1:1" ht="48" customHeight="1">
       <c r="A41" s="13" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="48" customHeight="1">
       <c r="A42" s="11" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="60" customHeight="1">
       <c r="A43" s="11" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="48" customHeight="1">
       <c r="A44" s="11" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="51.75" customHeight="1">
       <c r="A45" s="11" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -3779,61 +4545,61 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1">
       <c r="A5" s="62" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C5" s="4">
         <v>5</v>
       </c>
       <c r="D5" s="61" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1">
       <c r="A6" s="62" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="C6" s="4">
         <v>5</v>
       </c>
       <c r="D6" s="61" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1">
       <c r="A7" s="62" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="C7" s="4">
         <v>2.25</v>
       </c>
       <c r="D7" s="61" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="84" customHeight="1">
       <c r="A8" s="62" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="C8" s="4">
         <v>1.25</v>
       </c>
       <c r="D8" s="61" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1">
@@ -3841,31 +4607,31 @@
         <v>117</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="F9" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="H9" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>432</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>435</v>
-      </c>
       <c r="J9" s="5" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>17</v>
@@ -4197,17 +4963,17 @@
     </row>
     <row r="23" spans="1:11" ht="108" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="84" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="84" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="120" customHeight="1">
@@ -4215,27 +4981,27 @@
     </row>
     <row r="27" spans="1:11" ht="96" customHeight="1">
       <c r="A27" s="11" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="108" customHeight="1">
       <c r="A28" s="11" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="108" customHeight="1">
       <c r="A29" s="11" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="156" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="96" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -4256,126 +5022,126 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1">
       <c r="A1" s="64" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" s="56" t="s">
         <v>450</v>
-      </c>
-      <c r="C6" s="56" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1">
       <c r="A8" s="65" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C8" s="66" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1">
       <c r="A9" s="65" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B9" s="65" t="s">
+        <v>454</v>
+      </c>
+      <c r="C9" s="66" t="s">
         <v>457</v>
-      </c>
-      <c r="C9" s="66" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C10" s="67" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C11" s="56" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="C12" s="56" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="24" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="24" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="36" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15" customHeight="1">
@@ -4383,47 +5149,47 @@
     </row>
     <row r="19" spans="1:1" ht="36" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="36" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="48" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="16.5" customHeight="1">
       <c r="A25" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="16.5" customHeight="1">
       <c r="A26" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="16.5" customHeight="1">
       <c r="A27" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="16.5" customHeight="1">
       <c r="A28" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="16.5" customHeight="1">
       <c r="A30" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -4447,185 +5213,185 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="68" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1">
       <c r="A6" s="69" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B6" s="70" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="D6" s="69" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E6" s="69">
         <v>0</v>
       </c>
       <c r="F6" s="71" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="D7" s="65" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="E7" s="7">
         <f>복귀_화_상체밀기!$E$10</f>
         <v>19</v>
       </c>
       <c r="F7" s="67" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1">
       <c r="A8" s="69" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B8" s="70" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E8" s="69">
         <v>0</v>
       </c>
       <c r="F8" s="71" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1">
       <c r="A9" s="69" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B9" s="70" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D9" s="69" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E9" s="69">
         <v>0</v>
       </c>
       <c r="F9" s="71" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
       <c r="A10" s="69" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B10" s="70" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D10" s="69" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E10" s="69">
         <v>0</v>
       </c>
       <c r="F10" s="71" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D11" s="65" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="E11" s="7">
         <f>복귀_토_하체!$E$10</f>
         <v>15</v>
       </c>
       <c r="F11" s="56" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="D12" s="65" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="E12" s="7">
         <f>복귀_일_등!$E$10</f>
         <v>13</v>
       </c>
       <c r="F12" s="56" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1">
       <c r="A13" s="35" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="35"/>
@@ -4638,27 +5404,27 @@
     </row>
     <row r="15" spans="1:6" ht="48" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="141" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="126" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="77.25" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="115.5" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1">
@@ -4666,32 +5432,32 @@
     </row>
     <row r="21" spans="1:1" ht="48" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="141" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="77.25" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="90" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="128.25" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="128.25" customHeight="1">
       <c r="A26" s="11" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="15" customHeight="1">
@@ -4699,27 +5465,27 @@
     </row>
     <row r="28" spans="1:1" ht="48" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="75" customHeight="1">
       <c r="A29" s="11" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="102.75" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="90" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="128.25" customHeight="1">
       <c r="A32" s="11" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>
@@ -4746,12 +5512,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -4791,7 +5557,7 @@
         <v>39</v>
       </c>
       <c r="D5" s="65" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="E5" s="65">
         <v>5</v>
@@ -4800,10 +5566,10 @@
         <v>22</v>
       </c>
       <c r="G5" s="66" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="H5" s="66" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -4811,7 +5577,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>39</v>
@@ -4826,10 +5592,10 @@
         <v>41</v>
       </c>
       <c r="G6" s="56" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="H6" s="56" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -4837,7 +5603,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="56" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>46</v>
@@ -4853,7 +5619,7 @@
       </c>
       <c r="G7" s="56"/>
       <c r="H7" s="56" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -4861,7 +5627,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="56" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>57</v>
@@ -4876,10 +5642,10 @@
         <v>34</v>
       </c>
       <c r="G8" s="56" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="H8" s="56" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -4887,7 +5653,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="56" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>53</v>
@@ -4902,10 +5668,10 @@
         <v>34</v>
       </c>
       <c r="G9" s="56" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="H9" s="56" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -4919,22 +5685,22 @@
     </row>
     <row r="12" spans="1:8" ht="32.25" customHeight="1">
       <c r="A12" s="12" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="278.25" customHeight="1">
       <c r="A13" s="11" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="237.75" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="237.75" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
     </row>
   </sheetData>
@@ -4961,12 +5727,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -5003,10 +5769,10 @@
         <v>88</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D5" s="65" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="E5" s="65">
         <v>3</v>
@@ -5015,10 +5781,10 @@
         <v>22</v>
       </c>
       <c r="G5" s="66" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="H5" s="66" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -5026,10 +5792,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>67</v>
@@ -5038,13 +5804,13 @@
         <v>3</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G6" s="56" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="H6" s="56" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -5052,10 +5818,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="56" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>67</v>
@@ -5067,10 +5833,10 @@
         <v>58</v>
       </c>
       <c r="G7" s="56" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="H7" s="56" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -5078,10 +5844,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="56" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>67</v>
@@ -5094,7 +5860,7 @@
       </c>
       <c r="G8" s="56"/>
       <c r="H8" s="56" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -5108,7 +5874,7 @@
         <v>21</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="E9" s="7">
         <v>3</v>
@@ -5117,10 +5883,10 @@
         <v>22</v>
       </c>
       <c r="G9" s="56" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="H9" s="56" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -5134,22 +5900,22 @@
     </row>
     <row r="12" spans="1:8" ht="76.5" customHeight="1">
       <c r="A12" s="12" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="265.5" customHeight="1">
       <c r="A13" s="11" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="293.25" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="276" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
     </row>
   </sheetData>
@@ -5176,12 +5942,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -5218,10 +5984,10 @@
         <v>90</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D5" s="58" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E5" s="65">
         <v>1</v>
@@ -5230,10 +5996,10 @@
         <v>22</v>
       </c>
       <c r="G5" s="66" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="H5" s="66" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -5241,10 +6007,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>67</v>
@@ -5256,10 +6022,10 @@
         <v>48</v>
       </c>
       <c r="G6" s="56" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="H6" s="56" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -5267,25 +6033,25 @@
         <v>3</v>
       </c>
       <c r="B7" s="56" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E7" s="7">
         <v>3</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="G7" s="56" t="s">
+        <v>555</v>
+      </c>
+      <c r="H7" s="56" t="s">
         <v>558</v>
-      </c>
-      <c r="H7" s="56" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -5293,10 +6059,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="56" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>67</v>
@@ -5308,10 +6074,10 @@
         <v>41</v>
       </c>
       <c r="G8" s="56" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="H8" s="56" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -5334,10 +6100,10 @@
         <v>34</v>
       </c>
       <c r="G9" s="56" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="H9" s="56" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -5351,22 +6117,22 @@
     </row>
     <row r="12" spans="1:8" ht="92.25" customHeight="1">
       <c r="A12" s="12" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="233.25" customHeight="1">
       <c r="A13" s="11" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="240" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="278.25" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" customHeight="1">
@@ -5374,22 +6140,22 @@
     </row>
     <row r="17" spans="1:1" ht="95.25" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="252.75" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="237.75" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="265.5" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
     </row>
   </sheetData>
@@ -5411,96 +6177,96 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="D5" s="67" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
+        <v>579</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="D6" s="56" t="s">
         <v>582</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>583</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>584</v>
-      </c>
-      <c r="D6" s="56" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
+        <v>583</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>584</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>585</v>
+      </c>
+      <c r="D7" s="56" t="s">
         <v>586</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>587</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>588</v>
-      </c>
-      <c r="D7" s="56" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1">
       <c r="A8" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>588</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>589</v>
+      </c>
+      <c r="D8" s="56" t="s">
         <v>590</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>591</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>592</v>
-      </c>
-      <c r="D8" s="56" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1">
       <c r="A9" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>592</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>593</v>
+      </c>
+      <c r="D9" s="56" t="s">
         <v>594</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>595</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>596</v>
-      </c>
-      <c r="D9" s="56" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1">
@@ -5508,13 +6274,13 @@
         <v>90</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1">
@@ -5522,52 +6288,52 @@
         <v>88</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="D11" s="56" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>601</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>602</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>603</v>
+      </c>
+      <c r="D12" s="56" t="s">
         <v>604</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>605</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>606</v>
-      </c>
-      <c r="D12" s="56" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="39" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="51.75" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="39" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="39" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1">
@@ -5575,12 +6341,12 @@
     </row>
     <row r="21" spans="1:1" ht="51.75" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="39" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15" customHeight="1">
@@ -5588,12 +6354,12 @@
     </row>
     <row r="24" spans="1:1" ht="51.75" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="39" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
   </sheetData>
@@ -5605,7 +6371,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -5653,7 +6419,7 @@
       <c r="B5" s="18"/>
       <c r="C5" s="21">
         <f>IF($C$4&lt;=2,$C$9,IF($C$4&lt;=4,$C$10,$C$11))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>135</v>
@@ -5693,38 +6459,38 @@
         <v>140</v>
       </c>
       <c r="C9" s="24">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>141</v>
+        <v>613</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16.5" customHeight="1">
       <c r="A10" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>143</v>
-      </c>
       <c r="C10" s="24">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>144</v>
+        <v>614</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16.5" customHeight="1">
       <c r="A11" s="25" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C11" s="24">
         <v>1</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1">
@@ -5735,7 +6501,7 @@
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B13" s="18"/>
       <c r="C13" s="18"/>
@@ -5743,7 +6509,7 @@
     </row>
     <row r="14" spans="1:4" ht="16.5" customHeight="1">
       <c r="A14" s="20" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
@@ -5751,7 +6517,7 @@
     </row>
     <row r="15" spans="1:4" ht="16.5" customHeight="1">
       <c r="A15" s="20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="18"/>
@@ -5759,7 +6525,7 @@
     </row>
     <row r="16" spans="1:4" ht="16.5" customHeight="1">
       <c r="A16" s="20" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="18"/>
@@ -5767,7 +6533,7 @@
     </row>
     <row r="17" spans="1:4" ht="16.5" customHeight="1">
       <c r="A17" s="20" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
@@ -5789,7 +6555,7 @@
     </row>
     <row r="20" spans="1:4" ht="16.5" customHeight="1">
       <c r="A20" s="20" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B20" s="18"/>
       <c r="C20" s="18"/>
@@ -5797,7 +6563,7 @@
     </row>
     <row r="21" spans="1:4" ht="16.5" customHeight="1">
       <c r="A21" s="20" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B21" s="18"/>
       <c r="C21" s="18"/>
@@ -5805,7 +6571,7 @@
     </row>
     <row r="22" spans="1:4" ht="16.5" customHeight="1">
       <c r="A22" s="20" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B22" s="18"/>
       <c r="C22" s="18"/>
@@ -5813,7 +6579,7 @@
     </row>
     <row r="23" spans="1:4" ht="16.5" customHeight="1">
       <c r="A23" s="20" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -5827,7 +6593,7 @@
     </row>
     <row r="25" spans="1:4" ht="15" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -5835,7 +6601,7 @@
     </row>
     <row r="26" spans="1:4" ht="16.5" customHeight="1">
       <c r="A26" s="20" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -5843,7 +6609,7 @@
     </row>
     <row r="27" spans="1:4" ht="16.5" customHeight="1">
       <c r="A27" s="20" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -5851,7 +6617,7 @@
     </row>
     <row r="28" spans="1:4" ht="16.5" customHeight="1">
       <c r="A28" s="20" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -5859,7 +6625,7 @@
     </row>
     <row r="29" spans="1:4" ht="16.5" customHeight="1">
       <c r="A29" s="20" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -5873,7 +6639,7 @@
     </row>
     <row r="31" spans="1:4" ht="16.5" customHeight="1">
       <c r="A31" s="20" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -5881,7 +6647,7 @@
     </row>
     <row r="32" spans="1:4" ht="16.5" customHeight="1">
       <c r="A32" s="20" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -5889,11 +6655,31 @@
     </row>
     <row r="33" spans="1:4" ht="16.5" customHeight="1">
       <c r="A33" s="20" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
       <c r="D33" s="18"/>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="74" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="74" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" s="74" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="74" t="s">
+        <v>618</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="27" type="noConversion"/>
@@ -5915,166 +6701,166 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>166</v>
+        <v>619</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1">
       <c r="A4" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="26" t="s">
         <v>167</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>169</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>170</v>
       </c>
       <c r="E4" s="26" t="s">
         <v>5</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
       <c r="A5" s="27" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C5" s="29" t="s">
         <v>67</v>
       </c>
       <c r="D5" s="28" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E5" s="27">
         <f>월_당기기A!$E$14</f>
         <v>26</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1">
       <c r="A6" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>176</v>
-      </c>
-      <c r="B6" s="28" t="s">
-        <v>177</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>179</v>
       </c>
       <c r="E6" s="27">
         <f>화_밀기A!$E$25</f>
         <v>24</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
       <c r="A7" s="27" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" s="28" t="s">
         <v>180</v>
-      </c>
-      <c r="B7" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="C7" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>183</v>
       </c>
       <c r="E7" s="27">
         <f>수_하체A!$E$22</f>
         <v>26</v>
       </c>
       <c r="F7" s="27" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1">
       <c r="A8" s="30" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>67</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E8" s="30">
         <f>목_당기기B!$E$13</f>
         <v>24</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1">
       <c r="A9" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>188</v>
+      </c>
+      <c r="D9" s="28" t="s">
         <v>189</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>191</v>
-      </c>
-      <c r="D9" s="28" t="s">
-        <v>192</v>
       </c>
       <c r="E9" s="27">
         <f>금_밀기B!$E$29</f>
         <v>29</v>
       </c>
       <c r="F9" s="27" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
       <c r="A10" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>191</v>
+      </c>
+      <c r="C10" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="28" t="s">
         <v>193</v>
-      </c>
-      <c r="B10" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>195</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>196</v>
       </c>
       <c r="E10" s="27">
         <f>토_하체B!$E$23</f>
         <v>24</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
       <c r="A11" s="30" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C11" s="32" t="s">
         <v>67</v>
@@ -6091,7 +6877,7 @@
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
       <c r="A12" s="34" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B12" s="35"/>
       <c r="C12" s="36"/>
@@ -6103,62 +6889,62 @@
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1">
       <c r="A14" s="13" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="89.25" customHeight="1">
       <c r="A15" s="37" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="76.5" customHeight="1">
       <c r="A16" s="37" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="38.25" customHeight="1">
       <c r="A17" s="37" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="114.75" customHeight="1">
       <c r="A18" s="37" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="16.5" customHeight="1">
       <c r="A19" s="38" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="16.5" customHeight="1">
       <c r="A20" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15" customHeight="1">
       <c r="A21" s="39" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15" customHeight="1">
       <c r="A22" s="38" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15" customHeight="1">
       <c r="A23" s="38" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15" customHeight="1">
       <c r="A24" s="38" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="16.5" customHeight="1">
       <c r="A25" s="38" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="15" customHeight="1">
@@ -6166,27 +6952,27 @@
     </row>
     <row r="27" spans="1:1" ht="15" customHeight="1">
       <c r="A27" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="79.5" customHeight="1">
       <c r="A28" s="37" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="64.5" customHeight="1">
       <c r="A29" s="37" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="90" customHeight="1">
       <c r="A30" s="37" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="102.75" customHeight="1">
       <c r="A31" s="37" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="100.5" customHeight="1">
@@ -6194,17 +6980,17 @@
     </row>
     <row r="33" spans="1:1" ht="15" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="90" customHeight="1">
       <c r="A34" s="40" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="51.75" customHeight="1">
       <c r="A35" s="40" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="77.25" customHeight="1">
@@ -6212,22 +6998,22 @@
     </row>
     <row r="37" spans="1:1" ht="64.5" customHeight="1">
       <c r="A37" s="13" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="16.5" customHeight="1">
       <c r="A38" s="38" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="16.5" customHeight="1">
       <c r="A39" s="38" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="16.5" customHeight="1">
       <c r="A40" s="38" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -6256,12 +7042,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1">
@@ -6306,32 +7092,32 @@
         <v>1</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D6" s="27" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E6" s="27">
         <v>4</v>
       </c>
       <c r="F6" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="H6" s="28" t="s">
+        <v>229</v>
+      </c>
+      <c r="I6" s="28" t="s">
         <v>230</v>
-      </c>
-      <c r="G6" s="28" t="s">
-        <v>231</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>232</v>
-      </c>
-      <c r="I6" s="28" t="s">
-        <v>233</v>
       </c>
       <c r="J6" s="43">
         <f>MAX(1,ROUND(E6*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16.5" customHeight="1">
@@ -6339,10 +7125,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D7" s="33" t="s">
         <v>67</v>
@@ -6354,17 +7140,17 @@
         <v>41</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I7" s="28" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="J7" s="43">
         <f>MAX(1,ROUND(E7*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1">
@@ -6372,13 +7158,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C8" s="27" t="s">
         <v>32</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E8" s="27">
         <v>3</v>
@@ -6390,14 +7176,14 @@
         <v>35</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="J8" s="43">
         <f>MAX(1,ROUND(E8*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="16.5" customHeight="1">
@@ -6405,13 +7191,13 @@
         <v>4</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E9" s="27">
         <v>3</v>
@@ -6420,17 +7206,17 @@
         <v>41</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J9" s="43">
         <f>MAX(1,ROUND(E9*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="16.5" customHeight="1">
@@ -6438,10 +7224,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D10" s="33" t="s">
         <v>58</v>
@@ -6453,17 +7239,17 @@
         <v>41</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H10" s="28" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="I10" s="28" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="J10" s="43">
         <f>MAX(1,ROUND(E10*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="16.5" customHeight="1">
@@ -6471,10 +7257,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D11" s="27">
         <v>10</v>
@@ -6483,18 +7269,18 @@
         <v>4</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="G11" s="28"/>
       <c r="H11" s="28" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J11" s="43">
         <f>MAX(1,ROUND(E11*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
@@ -6502,30 +7288,30 @@
         <v>7</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D12" s="27" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E12" s="27">
         <v>3</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G12" s="28"/>
       <c r="H12" s="28" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="I12" s="28" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J12" s="43">
         <f>MAX(1,ROUND(E12*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1">
@@ -6533,10 +7319,10 @@
         <v>8</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D13" s="27">
         <v>20</v>
@@ -6548,17 +7334,17 @@
         <v>27</v>
       </c>
       <c r="G13" s="28" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="H13" s="28" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="I13" s="28" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="J13" s="43">
         <f>MAX(1,ROUND(E13*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1">
@@ -6571,7 +7357,7 @@
       </c>
       <c r="J14" s="46">
         <f>SUM(J6:J13)</f>
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -6600,17 +7386,17 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="16.5" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" customHeight="1">
@@ -6751,7 +7537,7 @@
         <v>1</v>
       </c>
       <c r="B20" s="49" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C20" s="50" t="s">
         <v>39</v>
@@ -6770,14 +7556,14 @@
         <v>49</v>
       </c>
       <c r="H20" s="49" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="I20" s="49" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="J20" s="52">
         <f>MAX(1,ROUND(E20*볼륨램프!$C$5,0))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="16.5" customHeight="1">
@@ -6785,13 +7571,13 @@
         <v>2</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C21" s="27" t="s">
         <v>39</v>
       </c>
       <c r="D21" s="27" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E21" s="27">
         <v>4</v>
@@ -6803,14 +7589,14 @@
         <v>42</v>
       </c>
       <c r="H21" s="28" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="I21" s="28" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="J21" s="43">
         <f>MAX(1,ROUND(E21*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="16.5" customHeight="1">
@@ -6818,7 +7604,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C22" s="27" t="s">
         <v>46</v>
@@ -6834,14 +7620,14 @@
       </c>
       <c r="G22" s="28"/>
       <c r="H22" s="28" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="I22" s="28" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="J22" s="43">
         <f>MAX(1,ROUND(E22*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="16.5" customHeight="1">
@@ -6849,13 +7635,13 @@
         <v>4</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C23" s="27" t="s">
         <v>42</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E23" s="27">
         <v>4</v>
@@ -6865,14 +7651,14 @@
       </c>
       <c r="G23" s="28"/>
       <c r="H23" s="28" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="I23" s="28" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="J23" s="43">
         <f>MAX(1,ROUND(E23*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="16.5" customHeight="1">
@@ -6880,7 +7666,7 @@
         <v>5</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C24" s="27" t="s">
         <v>57</v>
@@ -6896,14 +7682,14 @@
       </c>
       <c r="G24" s="28"/>
       <c r="H24" s="28" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I24" s="28" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="J24" s="43">
         <f>MAX(1,ROUND(E24*볼륨램프!$C$5,0))</f>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15" customHeight="1">
@@ -6916,7 +7702,7 @@
       </c>
       <c r="J25" s="43">
         <f>SUM(J20:J24)</f>
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -6945,17 +7731,17 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="16.5" customHeight="1">
@@ -7076,10 +7862,10 @@
         <v>1</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D15" s="51">
         <f>시작중량_설정!$E$7</f>
@@ -7092,17 +7878,17 @@
         <v>22</v>
       </c>
       <c r="G15" s="49" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="H15" s="49" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="I15" s="49" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="J15" s="52">
         <f>MAX(1,ROUND(E15*볼륨램프!$C$5,0))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="16.5" customHeight="1">
@@ -7110,10 +7896,10 @@
         <v>2</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D16" s="33" t="s">
         <v>67</v>
@@ -7125,17 +7911,17 @@
         <v>41</v>
       </c>
       <c r="G16" s="28" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="H16" s="28" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I16" s="28" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="J16" s="43">
         <f>MAX(1,ROUND(E16*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16.5" customHeight="1">
@@ -7143,10 +7929,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D17" s="27">
         <v>15</v>
@@ -7155,20 +7941,20 @@
         <v>3</v>
       </c>
       <c r="F17" s="33" t="s">
+        <v>290</v>
+      </c>
+      <c r="G17" s="28" t="s">
+        <v>291</v>
+      </c>
+      <c r="H17" s="28" t="s">
+        <v>292</v>
+      </c>
+      <c r="I17" s="28" t="s">
         <v>293</v>
-      </c>
-      <c r="G17" s="28" t="s">
-        <v>294</v>
-      </c>
-      <c r="H17" s="28" t="s">
-        <v>295</v>
-      </c>
-      <c r="I17" s="28" t="s">
-        <v>296</v>
       </c>
       <c r="J17" s="43">
         <f>MAX(1,ROUND(E17*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="16.5" customHeight="1">
@@ -7176,10 +7962,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D18" s="33" t="s">
         <v>67</v>
@@ -7192,14 +7978,14 @@
       </c>
       <c r="G18" s="28"/>
       <c r="H18" s="28" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="I18" s="28" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="J18" s="43">
         <f>MAX(1,ROUND(E18*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="16.5" customHeight="1">
@@ -7207,10 +7993,10 @@
         <v>5</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D19" s="33" t="s">
         <v>67</v>
@@ -7223,14 +8009,14 @@
       </c>
       <c r="G19" s="28"/>
       <c r="H19" s="28" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="I19" s="28" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J19" s="43">
         <f>MAX(1,ROUND(E19*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="16.5" customHeight="1">
@@ -7238,10 +8024,10 @@
         <v>6</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D20" s="33" t="s">
         <v>67</v>
@@ -7254,14 +8040,14 @@
       </c>
       <c r="G20" s="28"/>
       <c r="H20" s="28" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="I20" s="28" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="J20" s="43">
         <f>MAX(1,ROUND(E20*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="16.5" customHeight="1">
@@ -7269,10 +8055,10 @@
         <v>7</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D21" s="33" t="s">
         <v>67</v>
@@ -7281,18 +8067,18 @@
         <v>2</v>
       </c>
       <c r="F21" s="33" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="G21" s="28"/>
       <c r="H21" s="28" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="I21" s="28" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="J21" s="43">
         <f>MAX(1,ROUND(E21*볼륨램프!$C$5,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="15" customHeight="1">
@@ -7305,7 +8091,7 @@
       </c>
       <c r="J22" s="43">
         <f>SUM(J15:J21)</f>
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -7334,12 +8120,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1">
@@ -7384,10 +8170,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D6" s="33" t="s">
         <v>67</v>
@@ -7399,17 +8185,17 @@
         <v>48</v>
       </c>
       <c r="G6" s="28" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="H6" s="28" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="I6" s="28" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="J6" s="43">
         <f>MAX(1,ROUND(E6*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="16.5" customHeight="1">
@@ -7417,10 +8203,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D7" s="33" t="s">
         <v>67</v>
@@ -7432,17 +8218,17 @@
         <v>41</v>
       </c>
       <c r="G7" s="28" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="H7" s="28" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="I7" s="28" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="J7" s="43">
         <f>MAX(1,ROUND(E7*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1">
@@ -7450,13 +8236,13 @@
         <v>3</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E8" s="27">
         <v>3</v>
@@ -7468,14 +8254,14 @@
         <v>63</v>
       </c>
       <c r="H8" s="28" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="I8" s="28" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="J8" s="43">
         <f>MAX(1,ROUND(E8*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="16.5" customHeight="1">
@@ -7483,7 +8269,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>53</v>
@@ -7498,17 +8284,17 @@
         <v>27</v>
       </c>
       <c r="G9" s="28" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="H9" s="28" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="J9" s="43">
         <f>MAX(1,ROUND(E9*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="16.5" customHeight="1">
@@ -7516,13 +8302,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E10" s="27">
         <v>3</v>
@@ -7531,17 +8317,17 @@
         <v>41</v>
       </c>
       <c r="G10" s="28" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H10" s="28" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I10" s="29" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="J10" s="43">
         <f>MAX(1,ROUND(E10*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="16.5" customHeight="1">
@@ -7549,10 +8335,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D11" s="27">
         <v>10</v>
@@ -7561,18 +8347,18 @@
         <v>4</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="G11" s="28"/>
       <c r="H11" s="28" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I11" s="28" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="J11" s="43">
         <f>MAX(1,ROUND(E11*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
@@ -7580,10 +8366,10 @@
         <v>7</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D12" s="27">
         <v>2.5</v>
@@ -7596,14 +8382,14 @@
       </c>
       <c r="G12" s="28"/>
       <c r="H12" s="28" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="I12" s="28" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="J12" s="43">
         <f>MAX(1,ROUND(E12*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="15" customHeight="1">
@@ -7616,7 +8402,7 @@
       </c>
       <c r="J13" s="43">
         <f>SUM(J6:J12)</f>
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -7822,7 +8608,7 @@
       </c>
       <c r="J20" s="52">
         <f>MAX(1,ROUND(E20*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="16.5" customHeight="1">
@@ -7855,7 +8641,7 @@
       </c>
       <c r="J21" s="43">
         <f>MAX(1,ROUND(E21*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="16.5" customHeight="1">
@@ -7888,7 +8674,7 @@
       </c>
       <c r="J22" s="43">
         <f>MAX(1,ROUND(E22*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="16.5" customHeight="1">
@@ -7921,7 +8707,7 @@
       </c>
       <c r="J23" s="43">
         <f>MAX(1,ROUND(E23*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="16.5" customHeight="1">
@@ -7954,7 +8740,7 @@
       </c>
       <c r="J24" s="43">
         <f>MAX(1,ROUND(E24*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="16.5" customHeight="1">
@@ -7985,7 +8771,7 @@
       </c>
       <c r="J25" s="43">
         <f>MAX(1,ROUND(E25*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="16.5" customHeight="1">
@@ -8016,7 +8802,7 @@
       </c>
       <c r="J26" s="43">
         <f>MAX(1,ROUND(E26*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="16.5" customHeight="1">
@@ -8049,7 +8835,7 @@
       </c>
       <c r="J27" s="43">
         <f>MAX(1,ROUND(E27*볼륨램프!$C$5,0))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" customHeight="1">
@@ -8080,7 +8866,7 @@
       </c>
       <c r="J28" s="43">
         <f>MAX(1,ROUND(E28*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -8093,7 +8879,7 @@
       </c>
       <c r="J29" s="46">
         <f>SUM(J20:J28)</f>
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -8162,17 +8948,17 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.5" customHeight="1">
       <c r="A2" s="18" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="16.5" customHeight="1">
@@ -8293,10 +9079,10 @@
         <v>1</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D15" s="51">
         <f>시작중량_설정!$E$8</f>
@@ -8309,13 +9095,13 @@
         <v>22</v>
       </c>
       <c r="G15" s="49" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="H15" s="49" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="I15" s="49" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="J15" s="52">
         <f>MAX(1,ROUND(E15*볼륨램프!$C$5,0))</f>
@@ -8327,13 +9113,13 @@
         <v>2</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E16" s="27">
         <v>4</v>
@@ -8342,17 +9128,17 @@
         <v>41</v>
       </c>
       <c r="G16" s="28" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="H16" s="28" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="I16" s="28" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="J16" s="43">
         <f>MAX(1,ROUND(E16*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16.5" customHeight="1">
@@ -8360,10 +9146,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D17" s="27">
         <v>70</v>
@@ -8372,20 +9158,20 @@
         <v>3</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="G17" s="28" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="H17" s="28" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="I17" s="28" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="J17" s="43">
         <f>MAX(1,ROUND(E17*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="16.5" customHeight="1">
@@ -8393,10 +9179,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C18" s="27" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D18" s="33" t="s">
         <v>67</v>
@@ -8405,18 +9191,18 @@
         <v>3</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="G18" s="28"/>
       <c r="H18" s="28" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="I18" s="28" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="J18" s="43">
         <f>MAX(1,ROUND(E18*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="16.5" customHeight="1">
@@ -8424,10 +9210,10 @@
         <v>5</v>
       </c>
       <c r="B19" s="28" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D19" s="33" t="s">
         <v>67</v>
@@ -8440,14 +9226,14 @@
       </c>
       <c r="G19" s="28"/>
       <c r="H19" s="28" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="I19" s="28" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="J19" s="43">
         <f>MAX(1,ROUND(E19*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="16.5" customHeight="1">
@@ -8455,10 +9241,10 @@
         <v>6</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="D20" s="33" t="s">
         <v>67</v>
@@ -8467,18 +9253,18 @@
         <v>3</v>
       </c>
       <c r="F20" s="33" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G20" s="28"/>
       <c r="H20" s="28" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="I20" s="28" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="J20" s="43">
         <f>MAX(1,ROUND(E20*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="16.5" customHeight="1">
@@ -8486,10 +9272,10 @@
         <v>7</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D21" s="33" t="s">
         <v>67</v>
@@ -8502,14 +9288,14 @@
       </c>
       <c r="G21" s="28"/>
       <c r="H21" s="28" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="I21" s="28" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="J21" s="43">
         <f>MAX(1,ROUND(E21*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="16.5" customHeight="1">
@@ -8517,10 +9303,10 @@
         <v>8</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C22" s="27" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D22" s="33" t="s">
         <v>67</v>
@@ -8529,18 +9315,18 @@
         <v>3</v>
       </c>
       <c r="F22" s="33" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="G22" s="28"/>
       <c r="H22" s="28" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="I22" s="28" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="J22" s="43">
         <f>MAX(1,ROUND(E22*볼륨램프!$C$5,0))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="16.5" customHeight="1">
@@ -8553,7 +9339,7 @@
       </c>
       <c r="J23" s="43">
         <f>SUM(J15:J22)</f>
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="15" customHeight="1"/>

</xml_diff>